<commit_message>
Add new models Fix trends units Ensure dask and zarr chunks are aligned.
</commit_message>
<xml_diff>
--- a/scripts/eerie_menus.xlsx
+++ b/scripts/eerie_menus.xlsx
@@ -486,12 +486,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -527,12 +527,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -568,12 +568,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -613,12 +613,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -699,12 +699,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -740,12 +740,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -785,12 +785,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -830,12 +830,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -871,12 +871,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -912,12 +912,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -957,12 +957,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1174,12 +1174,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1215,12 +1215,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1256,12 +1256,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1301,12 +1301,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-mediumres', 'hadgem3-hires', 'hadgem3-lowres']</t>
+          <t>['ifs-fesom', 'icon', 'ifs-nemo-er', 'hadgem3-hires', 'hadgem3-lowres']</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin']</t>
+          <t>['sfcWind', 'uas', 'vas', 'tas', 'pr', 'tos', 'clt', 'zos', 'tasmax', 'tasmin', 'eke']</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">

</xml_diff>